<commit_message>
Cliente sin registrar, gatos y raza escrita, corbatín y moños en la ficha
- Nuevo turno: «Cliente nuevo» agenda solo con nombre, celular y mascota.
  El registro (cédula, dirección y consentimientos) se completa al llegar;
  sin él no se inicia la atención. Si la cédula ya existía, el cliente se
  une a ese propietario con sus mascotas, turnos y fichas.
- Mascotas: especie perro o gato, raza de la lista o escrita a mano (se
  agrega al catálogo sin tamaño). Raza «Gato (sin raza definida)».
- Ficha de servicio: corbatín y moños en las orejas, con su color.
- Migración 4, plantilla de Excel, pruebas, README, manual y resumen.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_012mAnuqmeJeeZZsZV8qRYdb
</commit_message>
<xml_diff>
--- a/plantilla_importacion.xlsx
+++ b/plantilla_importacion.xlsx
@@ -8,7 +8,7 @@
   </bookViews>
   <sheets>
     <sheet name="Mascotas" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Razas" sheetId="2" state="hidden" r:id="rId2"/>
+    <sheet name="Razas" sheetId="2" state="visible" r:id="rId2"/>
     <sheet name="Instrucciones" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
@@ -19,7 +19,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="4">
+  <fonts count="3">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -29,15 +29,10 @@
     </font>
     <font>
       <b val="1"/>
-      <color rgb="0014121D"/>
-      <sz val="12"/>
     </font>
     <font>
       <b val="1"/>
-      <sz val="12"/>
-    </font>
-    <font>
-      <sz val="12"/>
+      <sz val="14"/>
     </font>
   </fonts>
   <fills count="3">
@@ -65,13 +60,10 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -455,7 +447,7 @@
     <col width="40" customWidth="1" min="13" max="13"/>
   </cols>
   <sheetData>
-    <row r="1" ht="45" customHeight="1">
+    <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
           <t>Cédula del propietario *</t>
@@ -525,7 +517,7 @@
   </sheetData>
   <dataValidations count="3">
     <dataValidation sqref="G2:G2000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>=Razas!$A$1:$A$13</formula1>
+      <formula1>=Razas!$A$1:$A$14</formula1>
     </dataValidation>
     <dataValidation sqref="H2:H2000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Pequeña,Mediana,Grande"</formula1>
@@ -544,7 +536,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A13"/>
+  <dimension ref="A1:A14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -564,75 +556,82 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Golden Retriever</t>
+          <t>Gato (sin raza definida)</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Husky</t>
+          <t>Golden Retriever</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Labrador Retriever</t>
+          <t>Husky</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Pastor Alemán</t>
+          <t>Labrador Retriever</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Perro mestizo (sin raza)</t>
+          <t>Pastor Alemán</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Pitbull y similares</t>
+          <t>Perro mestizo (sin raza)</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Poodle (Caniche) Toy y Miniatura</t>
+          <t>Pitbull y similares</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Schnauzer</t>
+          <t>Poodle (Caniche) Toy y Miniatura</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Schnauzer Miniatura</t>
+          <t>Schnauzer</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Shih Tzu</t>
+          <t>Schnauzer Miniatura</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
+        <is>
+          <t>Shih Tzu</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
         <is>
           <t>Yorkshire Terrier</t>
         </is>
@@ -662,77 +661,73 @@
         </is>
       </c>
     </row>
-    <row r="2">
-      <c r="A2" s="3" t="inlineStr"/>
-    </row>
+    <row r="2"/>
     <row r="3">
-      <c r="A3" s="3" t="inlineStr">
+      <c r="A3" t="inlineStr">
         <is>
           <t>• Una fila por mascota. Si un propietario tiene varias mascotas, repita su cédula en cada fila.</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="3" t="inlineStr">
+      <c r="A4" t="inlineStr">
         <is>
           <t>• Las columnas con * son obligatorias.</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="3" t="inlineStr">
+      <c r="A5" t="inlineStr">
         <is>
           <t>• Raza: elija de la lista. Si la raza no existe, primero agréguela en Configuración › Razas.</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="3" t="inlineStr">
+      <c r="A6" t="inlineStr">
         <is>
           <t>• Tamaño: obligatorio para perros mestizos. En las demás razas, déjelo vacío para usar el de la raza.</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="3" t="inlineStr">
+      <c r="A7" t="inlineStr">
         <is>
           <t>• Pelaje complicado: obligatorio para perros mestizos (Sí o No).</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="3" t="inlineStr">
+      <c r="A8" t="inlineStr">
         <is>
           <t>• Fecha de última visita: formato AAAA-MM-DD (por ejemplo 2026-03-26) o como fecha de Excel.</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="3" t="inlineStr">
+      <c r="A9" t="inlineStr">
         <is>
           <t>• Si la cédula ya existe en el sistema, la mascota se agrega a ese propietario (sus datos no se cambian).</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="3" t="inlineStr">
+      <c r="A10" t="inlineStr">
         <is>
           <t>• Los consentimientos NO se importan: cada propietario debe aceptarlos antes de su primer turno.</t>
         </is>
       </c>
     </row>
-    <row r="11">
-      <c r="A11" s="3" t="inlineStr"/>
-    </row>
+    <row r="11"/>
     <row r="12">
-      <c r="A12" s="3" t="inlineStr">
+      <c r="A12" t="inlineStr">
         <is>
           <t>Ejemplo de fila:</t>
         </is>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="3" t="inlineStr">
+      <c r="A13" t="inlineStr">
         <is>
           <t>1098765432 | María Pérez | 3001234567 | | Calle 10 # 5-20 | Toby | Shih Tzu | | | 3 | 0 | 2026-02-15 | Nervioso con el secador</t>
         </is>

</xml_diff>